<commit_message>
Fixed some bugs with Digel and Messel, generated updated SLNs and collated into CompleteMetrics with run_all
e.g. Digel litter was considered an animal
</commit_message>
<xml_diff>
--- a/data/webinfo.xlsx
+++ b/data/webinfo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tannerfrank/Dropbox/Work/Devonian terr ecosystems/EcolNetworks/RhynieWebRepo/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5D6ACC0-A821-024D-AF73-38E668426832}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB975450-B2C7-A444-82E2-1133902F64E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="28800" windowHeight="16620" xr2:uid="{2FC7612B-5146-5244-858D-A0FBDE290E44}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1047" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1046" uniqueCount="242">
   <si>
     <t>dataset</t>
   </si>
@@ -1996,8 +1996,8 @@
       <c r="R15">
         <v>1</v>
       </c>
-      <c r="S15" t="s">
-        <v>149</v>
+      <c r="S15">
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.2">

</xml_diff>